<commit_message>
Remove redeemed Gridley parcel from Butte delivery package
APN 022-210-078-000 (Gridley Business Trust) was redeemed 2026-06-29,
confirmed against the county's own tax bill enricher output — the
delinquency was paid and the parcel is off the Aug 7-10 auction. It was
still being surfaced as the #1 "Level 1 Prime Opportunity" in last
night's regenerated dossiers, and was still physically present (just
low-ranked) in the combined PDF and XLSX in the existing Aug 2 delivery
package.

Pulled from every deliverable: the individual dossier PDF, the 208-page
combined PDF (now 206 pages, original backed up), the XLSX (Notes field
now explicitly flags REDEEMED — do not contact), and last night's
markdown dossier. The standalone summary PDF already correctly
documented this as a verification catch and needed no change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/butte/delivery/butte_auction_2026-08-02/butte_auction_intel_2026-08-02.xlsx
+++ b/butte/delivery/butte_auction_2026-08-02/butte_auction_intel_2026-08-02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc References" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Leads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Verification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Doc References" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to Use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -7531,9 +7530,7 @@
       <c r="L94" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M94" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M94" s="4" t="n"/>
       <c r="N94" s="5" t="n">
         <v>18</v>
       </c>
@@ -7602,9 +7599,7 @@
       <c r="L95" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M95" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M95" s="12" t="n"/>
       <c r="N95" s="13" t="n">
         <v>15</v>
       </c>
@@ -7661,9 +7656,7 @@
       <c r="L96" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M96" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M96" s="4" t="n"/>
       <c r="N96" s="5" t="n">
         <v>50</v>
       </c>
@@ -7736,9 +7729,7 @@
       <c r="L97" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M97" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M97" s="12" t="n"/>
       <c r="N97" s="13" t="n">
         <v>46</v>
       </c>
@@ -7811,9 +7802,7 @@
       <c r="L98" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M98" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M98" s="4" t="n"/>
       <c r="N98" s="5" t="n">
         <v>31</v>
       </c>
@@ -7870,9 +7859,7 @@
       <c r="L99" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M99" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M99" s="12" t="n"/>
       <c r="N99" s="13" t="n">
         <v>22</v>
       </c>
@@ -7941,9 +7928,7 @@
       <c r="L100" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M100" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M100" s="4" t="n"/>
       <c r="N100" s="5" t="n">
         <v>26</v>
       </c>
@@ -8004,9 +7989,7 @@
       <c r="L101" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M101" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M101" s="12" t="n"/>
       <c r="N101" s="13" t="n">
         <v>26</v>
       </c>
@@ -8075,9 +8058,7 @@
       <c r="L102" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M102" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M102" s="4" t="n"/>
       <c r="N102" s="5" t="n">
         <v>24</v>
       </c>
@@ -8134,9 +8115,7 @@
       <c r="L103" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M103" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M103" s="12" t="n"/>
       <c r="N103" s="13" t="n">
         <v>1</v>
       </c>
@@ -8197,9 +8176,7 @@
       <c r="L104" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="M104" s="4" t="n">
-        <v/>
-      </c>
+      <c r="M104" s="4" t="n"/>
       <c r="N104" s="5" t="n">
         <v>33</v>
       </c>
@@ -8260,9 +8237,7 @@
       <c r="L105" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M105" s="12" t="n">
-        <v/>
-      </c>
+      <c r="M105" s="12" t="n"/>
       <c r="N105" s="13" t="n">
         <v>10</v>
       </c>
@@ -8347,7 +8322,7 @@
       <c r="V106" s="3" t="inlineStr"/>
       <c r="W106" s="3" t="inlineStr">
         <is>
-          <t>Entity/Unparsed, skipped phone lookup</t>
+          <t>REDEEMED 2026-06-29 — delinquency paid, parcel OFF the auction. Do not contact. Kept in list only as verification proof.</t>
         </is>
       </c>
     </row>

</xml_diff>